<commit_message>
Add auto-highlight synchronization footer warning across MainWindow, SettingsDialog, and FirstRunDialog
</commit_message>
<xml_diff>
--- a/test_data.xlsx
+++ b/test_data.xlsx
@@ -2,23 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="FIR Records" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -29,16 +27,41 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -53,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -61,12 +84,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -430,17 +483,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I100"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="1" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -491,2615 +536,2615 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/101</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>1/26</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H2" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I2" s="2" t="n"/>
+      <c r="G2" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/102</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>2/26</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H3" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I3" s="2" t="n"/>
+      <c r="G3" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/103</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>3/26</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I4" s="2" t="n"/>
+      <c r="G4" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I4" s="4" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/104</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>4/26</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H5" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I5" s="2" t="n"/>
+      <c r="G5" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I5" s="4" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/105</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>5/26</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I6" s="2" t="n"/>
+      <c r="G6" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/106</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>6/26</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G7" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I7" s="2" t="n"/>
+      <c r="G7" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/107</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>7/26</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G8" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I8" s="2" t="n"/>
+      <c r="G8" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I8" s="4" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/108</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>8/26</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G9" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H9" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I9" s="2" t="n"/>
+      <c r="G9" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I9" s="4" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/109</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>9/26</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G10" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H10" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I10" s="2" t="n"/>
+      <c r="G10" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/110</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>10/26</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G11" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H11" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I11" s="2" t="n"/>
+      <c r="G11" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I11" s="4" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/111</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>11/26</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G12" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H12" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I12" s="2" t="n"/>
+      <c r="G12" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I12" s="4" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/112</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>12/26</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G13" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H13" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I13" s="2" t="n"/>
+      <c r="G13" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I13" s="4" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
+      <c r="A14" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/113</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>13/26</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G14" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H14" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I14" s="2" t="n"/>
+      <c r="G14" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I14" s="4" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
+      <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/114</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>14/26</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G15" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I15" s="2" t="n"/>
+      <c r="G15" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
+      <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/115</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>15/26</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G16" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H16" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I16" s="2" t="n"/>
+      <c r="G16" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
+      <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/116</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>16/26</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G17" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H17" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I17" s="2" t="n"/>
+      <c r="G17" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
+      <c r="A18" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/117</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>17/26</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G18" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H18" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I18" s="2" t="n"/>
+      <c r="G18" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
+      <c r="A19" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/118</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>18/26</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G19" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H19" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I19" s="2" t="n"/>
+      <c r="G19" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/119</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>19/26</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G20" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H20" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I20" s="2" t="n"/>
+      <c r="G20" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
+      <c r="A21" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/120</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>20/26</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G21" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H21" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I21" s="2" t="n"/>
+      <c r="G21" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/121</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>21/26</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G22" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H22" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I22" s="2" t="n"/>
+      <c r="G22" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
+      <c r="A23" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/122</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>22/26</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G23" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H23" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I23" s="2" t="n"/>
+      <c r="G23" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
+      <c r="A24" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/123</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>23/26</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G24" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H24" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I24" s="2" t="n"/>
+      <c r="G24" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/124</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>24/26</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G25" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H25" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I25" s="2" t="n"/>
+      <c r="G25" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
+      <c r="A26" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/125</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>25/26</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G26" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H26" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I26" s="2" t="n"/>
+      <c r="G26" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I26" s="4" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
+      <c r="A27" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/126</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>26/26</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G27" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H27" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I27" s="2" t="n"/>
+      <c r="G27" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I27" s="4" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
+      <c r="A28" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/127</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>27/26</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G28" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H28" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I28" s="2" t="n"/>
+      <c r="G28" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I28" s="4" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
+      <c r="A29" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/128</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>28/26</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G29" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H29" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I29" s="2" t="n"/>
+      <c r="G29" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I29" s="4" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
+      <c r="A30" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/129</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>29/26</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G30" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H30" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I30" s="2" t="n"/>
+      <c r="G30" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I30" s="4" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/130</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>30/26</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G31" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H31" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I31" s="2" t="n"/>
+      <c r="G31" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I31" s="4" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
+      <c r="A32" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/131</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>31/26</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G32" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H32" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I32" s="2" t="n"/>
+      <c r="G32" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I32" s="4" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
+      <c r="A33" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/132</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>32/26</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G33" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H33" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I33" s="2" t="n"/>
+      <c r="G33" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I33" s="4" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
+      <c r="A34" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/133</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>33/26</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G34" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H34" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I34" s="2" t="n"/>
+      <c r="G34" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I34" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
+      <c r="A35" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/134</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>34/26</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G35" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H35" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I35" s="2" t="n"/>
+      <c r="G35" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I35" s="4" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
+      <c r="A36" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/135</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>35/26</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G36" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H36" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I36" s="2" t="n"/>
+      <c r="G36" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H36" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I36" s="4" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
+      <c r="A37" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/136</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>36/26</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E37" s="4" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G37" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H37" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I37" s="2" t="n"/>
+      <c r="G37" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I37" s="4" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
+      <c r="A38" s="4" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/137</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>37/26</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G38" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H38" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I38" s="2" t="n"/>
+      <c r="G38" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I38" s="4" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
+      <c r="A39" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/138</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>38/26</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F39" s="4" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G39" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H39" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I39" s="2" t="n"/>
+      <c r="G39" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H39" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I39" s="4" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="4" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/139</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>39/26</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G40" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H40" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I40" s="2" t="n"/>
+      <c r="G40" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I40" s="4" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
+      <c r="A41" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/140</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>40/26</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G41" s="3" t="n">
+      <c r="G41" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H41" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I41" s="3" t="n">
+      <c r="H41" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I41" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/141</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>41/26</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G42" s="3" t="n">
+      <c r="G42" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H42" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I42" s="3" t="n">
+      <c r="H42" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I42" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
+      <c r="A43" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/142</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>42/26</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G43" s="3" t="n">
+      <c r="G43" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H43" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I43" s="3" t="n">
+      <c r="H43" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I43" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
+      <c r="A44" s="6" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/143</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C44" s="6" t="inlineStr">
         <is>
           <t>43/26</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E44" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F44" s="6" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G44" s="3" t="n">
+      <c r="G44" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H44" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I44" s="3" t="n">
+      <c r="H44" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I44" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
+      <c r="A45" s="6" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/144</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>44/26</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E45" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G45" s="3" t="n">
+      <c r="G45" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H45" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I45" s="3" t="n">
+      <c r="H45" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I45" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
+      <c r="A46" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/145</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>45/26</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E46" s="6" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G46" s="3" t="n">
+      <c r="G46" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H46" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I46" s="3" t="n">
+      <c r="H46" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I46" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
+      <c r="A47" s="6" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/146</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>46/26</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G47" s="3" t="n">
+      <c r="G47" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H47" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I47" s="3" t="n">
+      <c r="H47" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I47" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="6" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/147</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>47/26</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G48" s="3" t="n">
+      <c r="G48" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H48" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I48" s="3" t="n">
+      <c r="H48" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I48" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
+      <c r="A49" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/148</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>48/26</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E49" s="6" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G49" s="3" t="n">
+      <c r="G49" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H49" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I49" s="3" t="n">
+      <c r="H49" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I49" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
+      <c r="A50" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/149</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>49/26</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G50" s="3" t="n">
+      <c r="G50" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H50" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I50" s="3" t="n">
+      <c r="H50" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I50" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
+      <c r="A51" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/150</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>50/26</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E51" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G51" s="3" t="n">
+      <c r="G51" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H51" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I51" s="3" t="n">
+      <c r="H51" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I51" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
+      <c r="A52" s="6" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/151</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>51/26</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G52" s="3" t="n">
+      <c r="G52" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H52" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I52" s="3" t="n">
+      <c r="H52" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I52" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
+      <c r="A53" s="6" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/152</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>52/26</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E53" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G53" s="3" t="n">
+      <c r="G53" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H53" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I53" s="3" t="n">
+      <c r="H53" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I53" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="A54" s="6" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/153</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>53/26</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G54" s="3" t="n">
+      <c r="G54" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H54" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I54" s="3" t="n">
+      <c r="H54" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I54" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="A55" s="6" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/154</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>54/26</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G55" s="3" t="n">
+      <c r="G55" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H55" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I55" s="3" t="n">
+      <c r="H55" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I55" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="A56" s="6" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/155</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>55/26</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F56" s="6" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G56" s="3" t="n">
+      <c r="G56" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H56" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I56" s="3" t="n">
+      <c r="H56" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I56" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
+      <c r="A57" s="6" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/156</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>56/26</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E57" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F57" s="6" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G57" s="3" t="n">
+      <c r="G57" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H57" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I57" s="3" t="n">
+      <c r="H57" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I57" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
+      <c r="A58" s="6" t="n">
         <v>57</v>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/157</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>57/26</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G58" s="3" t="n">
+      <c r="G58" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H58" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I58" s="3" t="n">
+      <c r="H58" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I58" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
+      <c r="A59" s="6" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/158</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>58/26</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E59" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G59" s="3" t="n">
+      <c r="G59" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H59" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I59" s="3" t="n">
+      <c r="H59" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I59" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
+      <c r="A60" s="6" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B60" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/159</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr">
         <is>
           <t>59/26</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E60" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F60" s="6" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G60" s="3" t="n">
+      <c r="G60" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H60" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I60" s="3" t="n">
+      <c r="H60" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I60" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
+      <c r="A61" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B61" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/160</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C61" s="6" t="inlineStr">
         <is>
           <t>60/26</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D61" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E61" s="6" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F61" s="6" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G61" s="3" t="n">
+      <c r="G61" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H61" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I61" s="3" t="n">
+      <c r="H61" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I61" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
+      <c r="A62" s="6" t="n">
         <v>61</v>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B62" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/161</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C62" s="6" t="inlineStr">
         <is>
           <t>61/26</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D62" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E62" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F62" s="6" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G62" s="3" t="n">
+      <c r="G62" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H62" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I62" s="3" t="n">
+      <c r="H62" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I62" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
+      <c r="A63" s="6" t="n">
         <v>62</v>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B63" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/162</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C63" s="6" t="inlineStr">
         <is>
           <t>62/26</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D63" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E63" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="F63" s="6" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G63" s="3" t="n">
+      <c r="G63" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H63" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I63" s="3" t="n">
+      <c r="H63" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I63" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
+      <c r="A64" s="6" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B64" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/163</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C64" s="6" t="inlineStr">
         <is>
           <t>63/26</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="D64" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E64" s="6" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F64" s="6" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G64" s="3" t="n">
+      <c r="G64" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H64" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I64" s="3" t="n">
+      <c r="H64" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I64" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
+      <c r="A65" s="6" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B65" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/164</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C65" s="6" t="inlineStr">
         <is>
           <t>64/26</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D65" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E65" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F65" s="6" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G65" s="3" t="n">
+      <c r="G65" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H65" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I65" s="3" t="n">
+      <c r="H65" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I65" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n">
+      <c r="A66" s="6" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B66" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/165</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C66" s="6" t="inlineStr">
         <is>
           <t>65/26</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D66" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E66" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F66" s="6" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G66" s="3" t="n">
+      <c r="G66" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H66" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I66" s="3" t="n">
+      <c r="H66" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I66" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n">
+      <c r="A67" s="6" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B67" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/166</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
+      <c r="C67" s="6" t="inlineStr">
         <is>
           <t>66/26</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="D67" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E67" s="6" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F67" s="6" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G67" s="3" t="n">
+      <c r="G67" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H67" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I67" s="3" t="n">
+      <c r="H67" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I67" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n">
+      <c r="A68" s="6" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B68" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/167</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="C68" s="6" t="inlineStr">
         <is>
           <t>67/26</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="D68" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E68" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F68" s="6" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G68" s="3" t="n">
+      <c r="G68" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H68" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I68" s="3" t="n">
+      <c r="H68" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I68" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n">
+      <c r="A69" s="6" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B69" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/168</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C69" s="6" t="inlineStr">
         <is>
           <t>68/26</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="D69" s="6" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E69" s="6" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F69" s="6" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G69" s="3" t="n">
+      <c r="G69" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H69" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I69" s="3" t="n">
+      <c r="H69" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I69" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="6" t="n">
         <v>69</v>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B70" s="6" t="inlineStr">
         <is>
           <t>FSL/2026/169</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
+      <c r="C70" s="6" t="inlineStr">
         <is>
           <t>69/26</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="D70" s="6" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="E70" s="6" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr">
+      <c r="F70" s="6" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G70" s="3" t="n">
+      <c r="G70" s="7" t="n">
         <v>46130</v>
       </c>
-      <c r="H70" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I70" s="3" t="n">
+      <c r="H70" s="7" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I70" s="7" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3659,189 +3704,189 @@
       <c r="I85" s="2" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n">
+      <c r="A86" s="11" t="n">
         <v>85</v>
       </c>
-      <c r="B86" s="2" t="inlineStr">
+      <c r="B86" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/101</t>
         </is>
       </c>
-      <c r="C86" s="2" t="inlineStr">
+      <c r="C86" s="11" t="inlineStr">
         <is>
           <t>1/26</t>
         </is>
       </c>
-      <c r="D86" s="2" t="inlineStr">
+      <c r="D86" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E86" s="2" t="inlineStr">
+      <c r="E86" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F86" s="2" t="inlineStr">
+      <c r="F86" s="11" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G86" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H86" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I86" s="2" t="n"/>
+      <c r="G86" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H86" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I86" s="13" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n">
+      <c r="A87" s="4" t="n">
         <v>86</v>
       </c>
-      <c r="B87" s="2" t="inlineStr">
+      <c r="B87" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/102</t>
         </is>
       </c>
-      <c r="C87" s="2" t="inlineStr">
+      <c r="C87" s="4" t="inlineStr">
         <is>
           <t>2/26</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
+      <c r="D87" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E87" s="2" t="inlineStr">
+      <c r="E87" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F87" s="2" t="inlineStr">
+      <c r="F87" s="4" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G87" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H87" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I87" s="2" t="n"/>
+      <c r="G87" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H87" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I87" s="4" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n">
+      <c r="A88" s="4" t="n">
         <v>87</v>
       </c>
-      <c r="B88" s="2" t="inlineStr">
+      <c r="B88" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/103</t>
         </is>
       </c>
-      <c r="C88" s="2" t="inlineStr">
+      <c r="C88" s="4" t="inlineStr">
         <is>
           <t>3/26</t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr">
+      <c r="D88" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr">
+      <c r="E88" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr">
+      <c r="F88" s="4" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G88" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H88" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I88" s="2" t="n"/>
+      <c r="G88" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H88" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I88" s="4" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n">
+      <c r="A89" s="4" t="n">
         <v>88</v>
       </c>
-      <c r="B89" s="2" t="inlineStr">
+      <c r="B89" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/104</t>
         </is>
       </c>
-      <c r="C89" s="2" t="inlineStr">
+      <c r="C89" s="4" t="inlineStr">
         <is>
           <t>4/26</t>
         </is>
       </c>
-      <c r="D89" s="2" t="inlineStr">
+      <c r="D89" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E89" s="2" t="inlineStr">
+      <c r="E89" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F89" s="2" t="inlineStr">
+      <c r="F89" s="4" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G89" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H89" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I89" s="2" t="n"/>
+      <c r="G89" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H89" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I89" s="4" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n">
+      <c r="A90" s="4" t="n">
         <v>89</v>
       </c>
-      <c r="B90" s="2" t="inlineStr">
+      <c r="B90" s="4" t="inlineStr">
         <is>
           <t>FSL/2026/105</t>
         </is>
       </c>
-      <c r="C90" s="2" t="inlineStr">
+      <c r="C90" s="4" t="inlineStr">
         <is>
           <t>5/26</t>
         </is>
       </c>
-      <c r="D90" s="2" t="inlineStr">
+      <c r="D90" s="4" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E90" s="2" t="inlineStr">
+      <c r="E90" s="4" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr">
+      <c r="F90" s="4" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G90" s="3" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H90" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I90" s="2" t="n"/>
+      <c r="G90" s="5" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H90" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I90" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -3920,37 +3965,37 @@
       <c r="I95" s="2" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n">
+      <c r="A96" s="4" t="n">
         <v>93</v>
       </c>
-      <c r="B96" s="2" t="n"/>
-      <c r="C96" s="2" t="inlineStr">
+      <c r="B96" s="4" t="n"/>
+      <c r="C96" s="4" t="inlineStr">
         <is>
           <t>903/26</t>
         </is>
       </c>
-      <c r="D96" s="2" t="inlineStr">
+      <c r="D96" s="4" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E96" s="2" t="inlineStr">
+      <c r="E96" s="4" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F96" s="2" t="inlineStr">
+      <c r="F96" s="4" t="inlineStr">
         <is>
           <t>Officer Z</t>
         </is>
       </c>
-      <c r="G96" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="H96" s="3" t="n">
+      <c r="G96" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="H96" s="5" t="n">
         <v>46145</v>
       </c>
-      <c r="I96" s="2" t="n"/>
+      <c r="I96" s="4" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Optimize layout spacing and margins for highlight synchronization notes across all windows
</commit_message>
<xml_diff>
--- a/test_data.xlsx
+++ b/test_data.xlsx
@@ -32,7 +32,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +63,12 @@
         <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -76,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -115,6 +121,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -536,2615 +548,2615 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="n">
+      <c r="A2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/101</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>1/26</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G2" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H2" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I2" s="4" t="n"/>
+      <c r="G2" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H2" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I2" s="11" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/102</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>2/26</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H3" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I3" s="4" t="n"/>
+      <c r="G3" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H3" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I3" s="11" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/103</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>3/26</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I4" s="4" t="n"/>
+      <c r="G4" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H4" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I4" s="11" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/104</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>4/26</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H5" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I5" s="4" t="n"/>
+      <c r="G5" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H5" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I5" s="11" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/105</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>5/26</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G6" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I6" s="4" t="n"/>
+      <c r="G6" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H6" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I6" s="11" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/106</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>6/26</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G7" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I7" s="4" t="n"/>
+      <c r="G7" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/107</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>7/26</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G8" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I8" s="4" t="n"/>
+      <c r="G8" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H8" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/108</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>8/26</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G9" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H9" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I9" s="4" t="n"/>
+      <c r="G9" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H9" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/109</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>9/26</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G10" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H10" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I10" s="4" t="n"/>
+      <c r="G10" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H10" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/110</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>10/26</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G11" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I11" s="4" t="n"/>
+      <c r="G11" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H11" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/111</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>11/26</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G12" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H12" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I12" s="4" t="n"/>
+      <c r="G12" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H12" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/112</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>12/26</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G13" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H13" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I13" s="4" t="n"/>
+      <c r="G13" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H13" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/113</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>13/26</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="11" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G14" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H14" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I14" s="4" t="n"/>
+      <c r="G14" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H14" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n">
+      <c r="A15" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/114</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>14/26</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G15" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H15" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I15" s="4" t="n"/>
+      <c r="G15" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H15" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n">
+      <c r="A16" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/115</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>15/26</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="11" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G16" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H16" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I16" s="4" t="n"/>
+      <c r="G16" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H16" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="n">
+      <c r="A17" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/116</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>16/26</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F17" s="11" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G17" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H17" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I17" s="4" t="n"/>
+      <c r="G17" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H17" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="n">
+      <c r="A18" s="11" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/117</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>17/26</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G18" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H18" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I18" s="4" t="n"/>
+      <c r="G18" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H18" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/118</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>18/26</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F19" s="11" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G19" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H19" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I19" s="4" t="n"/>
+      <c r="G19" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H19" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I19" s="11" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="11" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/119</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>19/26</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F20" s="11" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G20" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H20" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I20" s="4" t="n"/>
+      <c r="G20" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H20" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I20" s="11" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/120</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>20/26</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G21" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H21" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I21" s="4" t="n"/>
+      <c r="G21" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H21" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I21" s="11" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n">
+      <c r="A22" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/121</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>21/26</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F22" s="11" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G22" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H22" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I22" s="4" t="n"/>
+      <c r="G22" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H22" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I22" s="11" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="n">
+      <c r="A23" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/122</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>22/26</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F23" s="11" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G23" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H23" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I23" s="4" t="n"/>
+      <c r="G23" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H23" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I23" s="11" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/123</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
         <is>
           <t>23/26</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F24" s="11" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G24" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H24" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I24" s="4" t="n"/>
+      <c r="G24" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H24" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I24" s="11" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="n">
+      <c r="A25" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/124</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>24/26</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F25" s="11" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G25" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H25" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I25" s="4" t="n"/>
+      <c r="G25" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H25" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I25" s="11" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/125</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>25/26</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F26" s="11" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G26" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H26" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I26" s="4" t="n"/>
+      <c r="G26" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H26" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I26" s="11" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="n">
+      <c r="A27" s="11" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/126</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>26/26</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="F27" s="11" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G27" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H27" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I27" s="4" t="n"/>
+      <c r="G27" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H27" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I27" s="11" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="n">
+      <c r="A28" s="11" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/127</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
         <is>
           <t>27/26</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F28" s="11" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G28" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H28" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I28" s="4" t="n"/>
+      <c r="G28" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H28" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I28" s="11" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="n">
+      <c r="A29" s="11" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/128</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>28/26</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G29" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H29" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I29" s="4" t="n"/>
+      <c r="G29" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H29" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I29" s="11" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="n">
+      <c r="A30" s="11" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/129</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>29/26</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="F30" s="11" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G30" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H30" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I30" s="4" t="n"/>
+      <c r="G30" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H30" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I30" s="11" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n">
+      <c r="A31" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/130</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>30/26</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E31" s="11" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F31" s="11" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G31" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H31" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I31" s="4" t="n"/>
+      <c r="G31" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H31" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I31" s="11" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="n">
+      <c r="A32" s="11" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/131</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>31/26</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F32" s="11" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G32" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H32" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I32" s="4" t="n"/>
+      <c r="G32" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H32" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I32" s="11" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="n">
+      <c r="A33" s="11" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/132</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
         <is>
           <t>32/26</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D33" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E33" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F33" s="11" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G33" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H33" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I33" s="4" t="n"/>
+      <c r="G33" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H33" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I33" s="11" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="n">
+      <c r="A34" s="11" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/133</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C34" s="11" t="inlineStr">
         <is>
           <t>33/26</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F34" s="11" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G34" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H34" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I34" s="4" t="n"/>
+      <c r="G34" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H34" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I34" s="11" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="n">
+      <c r="A35" s="11" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/134</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>34/26</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D35" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E35" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F35" s="11" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G35" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H35" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I35" s="4" t="n"/>
+      <c r="G35" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H35" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I35" s="11" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n">
+      <c r="A36" s="11" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/135</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>35/26</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D36" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F36" s="11" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G36" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H36" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I36" s="4" t="n"/>
+      <c r="G36" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H36" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I36" s="11" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="n">
+      <c r="A37" s="11" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/136</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
         <is>
           <t>36/26</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D37" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E37" s="11" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="F37" s="11" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G37" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H37" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I37" s="4" t="n"/>
+      <c r="G37" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H37" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I37" s="11" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="n">
+      <c r="A38" s="11" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/137</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C38" s="11" t="inlineStr">
         <is>
           <t>37/26</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D38" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F38" s="11" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G38" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H38" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I38" s="4" t="n"/>
+      <c r="G38" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H38" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I38" s="11" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="n">
+      <c r="A39" s="11" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/138</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>38/26</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D39" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E39" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="F39" s="11" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G39" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H39" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I39" s="4" t="n"/>
+      <c r="G39" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H39" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I39" s="11" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="n">
+      <c r="A40" s="11" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B40" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/139</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
         <is>
           <t>39/26</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="11" t="inlineStr">
         <is>
           <t>Kotwali PS</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>302 IPC</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="F40" s="11" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G40" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H40" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I40" s="4" t="n"/>
+      <c r="G40" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H40" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I40" s="11" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="n">
+      <c r="A41" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B41" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/140</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C41" s="14" t="inlineStr">
         <is>
           <t>40/26</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="D41" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="E41" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F41" s="6" t="inlineStr">
+      <c r="F41" s="14" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G41" s="7" t="n">
+      <c r="G41" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H41" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I41" s="7" t="n">
+      <c r="H41" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I41" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="n">
+      <c r="A42" s="14" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B42" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/141</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C42" s="14" t="inlineStr">
         <is>
           <t>41/26</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D42" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="E42" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F42" s="6" t="inlineStr">
+      <c r="F42" s="14" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G42" s="7" t="n">
+      <c r="G42" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H42" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I42" s="7" t="n">
+      <c r="H42" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I42" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="n">
+      <c r="A43" s="14" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/142</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="C43" s="14" t="inlineStr">
         <is>
           <t>42/26</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="D43" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E43" s="6" t="inlineStr">
+      <c r="E43" s="14" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="F43" s="14" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G43" s="7" t="n">
+      <c r="G43" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H43" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I43" s="7" t="n">
+      <c r="H43" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I43" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="n">
+      <c r="A44" s="14" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="6" t="inlineStr">
+      <c r="B44" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/143</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
+      <c r="C44" s="14" t="inlineStr">
         <is>
           <t>43/26</t>
         </is>
       </c>
-      <c r="D44" s="6" t="inlineStr">
+      <c r="D44" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E44" s="6" t="inlineStr">
+      <c r="E44" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F44" s="6" t="inlineStr">
+      <c r="F44" s="14" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G44" s="7" t="n">
+      <c r="G44" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H44" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I44" s="7" t="n">
+      <c r="H44" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I44" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="n">
+      <c r="A45" s="14" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="6" t="inlineStr">
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/144</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C45" s="14" t="inlineStr">
         <is>
           <t>44/26</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr">
+      <c r="D45" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E45" s="6" t="inlineStr">
+      <c r="E45" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F45" s="6" t="inlineStr">
+      <c r="F45" s="14" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G45" s="7" t="n">
+      <c r="G45" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H45" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I45" s="7" t="n">
+      <c r="H45" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I45" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="n">
+      <c r="A46" s="14" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B46" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/145</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C46" s="14" t="inlineStr">
         <is>
           <t>45/26</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D46" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
+      <c r="E46" s="14" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F46" s="6" t="inlineStr">
+      <c r="F46" s="14" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G46" s="7" t="n">
+      <c r="G46" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H46" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I46" s="7" t="n">
+      <c r="H46" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I46" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="n">
+      <c r="A47" s="14" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/146</t>
         </is>
       </c>
-      <c r="C47" s="6" t="inlineStr">
+      <c r="C47" s="14" t="inlineStr">
         <is>
           <t>46/26</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr">
+      <c r="D47" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E47" s="6" t="inlineStr">
+      <c r="E47" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F47" s="6" t="inlineStr">
+      <c r="F47" s="14" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G47" s="7" t="n">
+      <c r="G47" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H47" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I47" s="7" t="n">
+      <c r="H47" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I47" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="n">
+      <c r="A48" s="14" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="6" t="inlineStr">
+      <c r="B48" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/147</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C48" s="14" t="inlineStr">
         <is>
           <t>47/26</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="D48" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
+      <c r="E48" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F48" s="6" t="inlineStr">
+      <c r="F48" s="14" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G48" s="7" t="n">
+      <c r="G48" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H48" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I48" s="7" t="n">
+      <c r="H48" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I48" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="n">
+      <c r="A49" s="14" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="B49" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/148</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C49" s="14" t="inlineStr">
         <is>
           <t>48/26</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="D49" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
+      <c r="E49" s="14" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F49" s="6" t="inlineStr">
+      <c r="F49" s="14" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G49" s="7" t="n">
+      <c r="G49" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H49" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I49" s="7" t="n">
+      <c r="H49" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I49" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="n">
+      <c r="A50" s="14" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="6" t="inlineStr">
+      <c r="B50" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/149</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C50" s="14" t="inlineStr">
         <is>
           <t>49/26</t>
         </is>
       </c>
-      <c r="D50" s="6" t="inlineStr">
+      <c r="D50" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E50" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F50" s="6" t="inlineStr">
+      <c r="F50" s="14" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G50" s="7" t="n">
+      <c r="G50" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H50" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I50" s="7" t="n">
+      <c r="H50" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I50" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="n">
+      <c r="A51" s="14" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B51" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/150</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C51" s="14" t="inlineStr">
         <is>
           <t>50/26</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="D51" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E51" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F51" s="6" t="inlineStr">
+      <c r="F51" s="14" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G51" s="7" t="n">
+      <c r="G51" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H51" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I51" s="7" t="n">
+      <c r="H51" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I51" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="n">
+      <c r="A52" s="14" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B52" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/151</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C52" s="14" t="inlineStr">
         <is>
           <t>51/26</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
+      <c r="D52" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="E52" s="14" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr">
+      <c r="F52" s="14" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G52" s="7" t="n">
+      <c r="G52" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H52" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I52" s="7" t="n">
+      <c r="H52" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I52" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="n">
+      <c r="A53" s="14" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B53" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/152</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C53" s="14" t="inlineStr">
         <is>
           <t>52/26</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="D53" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="E53" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="F53" s="14" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G53" s="7" t="n">
+      <c r="G53" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H53" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I53" s="7" t="n">
+      <c r="H53" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I53" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="n">
+      <c r="A54" s="14" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B54" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/153</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C54" s="14" t="inlineStr">
         <is>
           <t>53/26</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
+      <c r="D54" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="E54" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr">
+      <c r="F54" s="14" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G54" s="7" t="n">
+      <c r="G54" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H54" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I54" s="7" t="n">
+      <c r="H54" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I54" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="n">
+      <c r="A55" s="14" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="6" t="inlineStr">
+      <c r="B55" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/154</t>
         </is>
       </c>
-      <c r="C55" s="6" t="inlineStr">
+      <c r="C55" s="14" t="inlineStr">
         <is>
           <t>54/26</t>
         </is>
       </c>
-      <c r="D55" s="6" t="inlineStr">
+      <c r="D55" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E55" s="6" t="inlineStr">
+      <c r="E55" s="14" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F55" s="6" t="inlineStr">
+      <c r="F55" s="14" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G55" s="7" t="n">
+      <c r="G55" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H55" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I55" s="7" t="n">
+      <c r="H55" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I55" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="n">
+      <c r="A56" s="14" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B56" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/155</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C56" s="14" t="inlineStr">
         <is>
           <t>55/26</t>
         </is>
       </c>
-      <c r="D56" s="6" t="inlineStr">
+      <c r="D56" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E56" s="6" t="inlineStr">
+      <c r="E56" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F56" s="6" t="inlineStr">
+      <c r="F56" s="14" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G56" s="7" t="n">
+      <c r="G56" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H56" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I56" s="7" t="n">
+      <c r="H56" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I56" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="n">
+      <c r="A57" s="14" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="6" t="inlineStr">
+      <c r="B57" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/156</t>
         </is>
       </c>
-      <c r="C57" s="6" t="inlineStr">
+      <c r="C57" s="14" t="inlineStr">
         <is>
           <t>56/26</t>
         </is>
       </c>
-      <c r="D57" s="6" t="inlineStr">
+      <c r="D57" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E57" s="6" t="inlineStr">
+      <c r="E57" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F57" s="6" t="inlineStr">
+      <c r="F57" s="14" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G57" s="7" t="n">
+      <c r="G57" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H57" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I57" s="7" t="n">
+      <c r="H57" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I57" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="n">
+      <c r="A58" s="14" t="n">
         <v>57</v>
       </c>
-      <c r="B58" s="6" t="inlineStr">
+      <c r="B58" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/157</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C58" s="14" t="inlineStr">
         <is>
           <t>57/26</t>
         </is>
       </c>
-      <c r="D58" s="6" t="inlineStr">
+      <c r="D58" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="E58" s="14" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F58" s="6" t="inlineStr">
+      <c r="F58" s="14" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G58" s="7" t="n">
+      <c r="G58" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H58" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I58" s="7" t="n">
+      <c r="H58" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I58" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="n">
+      <c r="A59" s="14" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="6" t="inlineStr">
+      <c r="B59" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/158</t>
         </is>
       </c>
-      <c r="C59" s="6" t="inlineStr">
+      <c r="C59" s="14" t="inlineStr">
         <is>
           <t>58/26</t>
         </is>
       </c>
-      <c r="D59" s="6" t="inlineStr">
+      <c r="D59" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E59" s="6" t="inlineStr">
+      <c r="E59" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F59" s="6" t="inlineStr">
+      <c r="F59" s="14" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G59" s="7" t="n">
+      <c r="G59" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H59" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I59" s="7" t="n">
+      <c r="H59" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I59" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="n">
+      <c r="A60" s="14" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B60" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/159</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C60" s="14" t="inlineStr">
         <is>
           <t>59/26</t>
         </is>
       </c>
-      <c r="D60" s="6" t="inlineStr">
+      <c r="D60" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E60" s="6" t="inlineStr">
+      <c r="E60" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F60" s="6" t="inlineStr">
+      <c r="F60" s="14" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G60" s="7" t="n">
+      <c r="G60" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H60" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I60" s="7" t="n">
+      <c r="H60" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I60" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="6" t="n">
+      <c r="A61" s="14" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="6" t="inlineStr">
+      <c r="B61" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/160</t>
         </is>
       </c>
-      <c r="C61" s="6" t="inlineStr">
+      <c r="C61" s="14" t="inlineStr">
         <is>
           <t>60/26</t>
         </is>
       </c>
-      <c r="D61" s="6" t="inlineStr">
+      <c r="D61" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E61" s="6" t="inlineStr">
+      <c r="E61" s="14" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F61" s="6" t="inlineStr">
+      <c r="F61" s="14" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G61" s="7" t="n">
+      <c r="G61" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H61" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I61" s="7" t="n">
+      <c r="H61" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I61" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="n">
+      <c r="A62" s="14" t="n">
         <v>61</v>
       </c>
-      <c r="B62" s="6" t="inlineStr">
+      <c r="B62" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/161</t>
         </is>
       </c>
-      <c r="C62" s="6" t="inlineStr">
+      <c r="C62" s="14" t="inlineStr">
         <is>
           <t>61/26</t>
         </is>
       </c>
-      <c r="D62" s="6" t="inlineStr">
+      <c r="D62" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E62" s="6" t="inlineStr">
+      <c r="E62" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F62" s="6" t="inlineStr">
+      <c r="F62" s="14" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G62" s="7" t="n">
+      <c r="G62" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H62" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I62" s="7" t="n">
+      <c r="H62" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I62" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="6" t="n">
+      <c r="A63" s="14" t="n">
         <v>62</v>
       </c>
-      <c r="B63" s="6" t="inlineStr">
+      <c r="B63" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/162</t>
         </is>
       </c>
-      <c r="C63" s="6" t="inlineStr">
+      <c r="C63" s="14" t="inlineStr">
         <is>
           <t>62/26</t>
         </is>
       </c>
-      <c r="D63" s="6" t="inlineStr">
+      <c r="D63" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E63" s="6" t="inlineStr">
+      <c r="E63" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F63" s="6" t="inlineStr">
+      <c r="F63" s="14" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G63" s="7" t="n">
+      <c r="G63" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H63" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I63" s="7" t="n">
+      <c r="H63" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I63" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="n">
+      <c r="A64" s="14" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="6" t="inlineStr">
+      <c r="B64" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/163</t>
         </is>
       </c>
-      <c r="C64" s="6" t="inlineStr">
+      <c r="C64" s="14" t="inlineStr">
         <is>
           <t>63/26</t>
         </is>
       </c>
-      <c r="D64" s="6" t="inlineStr">
+      <c r="D64" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E64" s="6" t="inlineStr">
+      <c r="E64" s="14" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F64" s="6" t="inlineStr">
+      <c r="F64" s="14" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G64" s="7" t="n">
+      <c r="G64" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H64" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I64" s="7" t="n">
+      <c r="H64" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I64" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="n">
+      <c r="A65" s="14" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="6" t="inlineStr">
+      <c r="B65" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/164</t>
         </is>
       </c>
-      <c r="C65" s="6" t="inlineStr">
+      <c r="C65" s="14" t="inlineStr">
         <is>
           <t>64/26</t>
         </is>
       </c>
-      <c r="D65" s="6" t="inlineStr">
+      <c r="D65" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E65" s="6" t="inlineStr">
+      <c r="E65" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F65" s="6" t="inlineStr">
+      <c r="F65" s="14" t="inlineStr">
         <is>
           <t>Officer E</t>
         </is>
       </c>
-      <c r="G65" s="7" t="n">
+      <c r="G65" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H65" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I65" s="7" t="n">
+      <c r="H65" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I65" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="n">
+      <c r="A66" s="14" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="6" t="inlineStr">
+      <c r="B66" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/165</t>
         </is>
       </c>
-      <c r="C66" s="6" t="inlineStr">
+      <c r="C66" s="14" t="inlineStr">
         <is>
           <t>65/26</t>
         </is>
       </c>
-      <c r="D66" s="6" t="inlineStr">
+      <c r="D66" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E66" s="6" t="inlineStr">
+      <c r="E66" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F66" s="6" t="inlineStr">
+      <c r="F66" s="14" t="inlineStr">
         <is>
           <t>Officer F</t>
         </is>
       </c>
-      <c r="G66" s="7" t="n">
+      <c r="G66" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H66" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I66" s="7" t="n">
+      <c r="H66" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I66" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="6" t="n">
+      <c r="A67" s="14" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="6" t="inlineStr">
+      <c r="B67" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/166</t>
         </is>
       </c>
-      <c r="C67" s="6" t="inlineStr">
+      <c r="C67" s="14" t="inlineStr">
         <is>
           <t>66/26</t>
         </is>
       </c>
-      <c r="D67" s="6" t="inlineStr">
+      <c r="D67" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E67" s="6" t="inlineStr">
+      <c r="E67" s="14" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F67" s="6" t="inlineStr">
+      <c r="F67" s="14" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G67" s="7" t="n">
+      <c r="G67" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H67" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I67" s="7" t="n">
+      <c r="H67" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I67" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="6" t="n">
+      <c r="A68" s="14" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="6" t="inlineStr">
+      <c r="B68" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/167</t>
         </is>
       </c>
-      <c r="C68" s="6" t="inlineStr">
+      <c r="C68" s="14" t="inlineStr">
         <is>
           <t>67/26</t>
         </is>
       </c>
-      <c r="D68" s="6" t="inlineStr">
+      <c r="D68" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E68" s="6" t="inlineStr">
+      <c r="E68" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F68" s="6" t="inlineStr">
+      <c r="F68" s="14" t="inlineStr">
         <is>
           <t>Officer B</t>
         </is>
       </c>
-      <c r="G68" s="7" t="n">
+      <c r="G68" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H68" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I68" s="7" t="n">
+      <c r="H68" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I68" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="6" t="n">
+      <c r="A69" s="14" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="6" t="inlineStr">
+      <c r="B69" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/168</t>
         </is>
       </c>
-      <c r="C69" s="6" t="inlineStr">
+      <c r="C69" s="14" t="inlineStr">
         <is>
           <t>68/26</t>
         </is>
       </c>
-      <c r="D69" s="6" t="inlineStr">
+      <c r="D69" s="14" t="inlineStr">
         <is>
           <t>Civil Lines PS</t>
         </is>
       </c>
-      <c r="E69" s="6" t="inlineStr">
+      <c r="E69" s="14" t="inlineStr">
         <is>
           <t>379 IPC</t>
         </is>
       </c>
-      <c r="F69" s="6" t="inlineStr">
+      <c r="F69" s="14" t="inlineStr">
         <is>
           <t>Officer C</t>
         </is>
       </c>
-      <c r="G69" s="7" t="n">
+      <c r="G69" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H69" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I69" s="7" t="n">
+      <c r="H69" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I69" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="6" t="n">
+      <c r="A70" s="14" t="n">
         <v>69</v>
       </c>
-      <c r="B70" s="6" t="inlineStr">
+      <c r="B70" s="14" t="inlineStr">
         <is>
           <t>FSL/2026/169</t>
         </is>
       </c>
-      <c r="C70" s="6" t="inlineStr">
+      <c r="C70" s="14" t="inlineStr">
         <is>
           <t>69/26</t>
         </is>
       </c>
-      <c r="D70" s="6" t="inlineStr">
+      <c r="D70" s="14" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E70" s="6" t="inlineStr">
+      <c r="E70" s="14" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F70" s="6" t="inlineStr">
+      <c r="F70" s="14" t="inlineStr">
         <is>
           <t>Officer D</t>
         </is>
       </c>
-      <c r="G70" s="7" t="n">
+      <c r="G70" s="15" t="n">
         <v>46130</v>
       </c>
-      <c r="H70" s="7" t="n">
-        <v>46135</v>
-      </c>
-      <c r="I70" s="7" t="n">
+      <c r="H70" s="15" t="n">
+        <v>46135</v>
+      </c>
+      <c r="I70" s="15" t="n">
         <v>46155</v>
       </c>
     </row>
@@ -3741,152 +3753,152 @@
       <c r="I86" s="13" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="4" t="n">
+      <c r="A87" s="11" t="n">
         <v>86</v>
       </c>
-      <c r="B87" s="4" t="inlineStr">
+      <c r="B87" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/102</t>
         </is>
       </c>
-      <c r="C87" s="4" t="inlineStr">
+      <c r="C87" s="11" t="inlineStr">
         <is>
           <t>2/26</t>
         </is>
       </c>
-      <c r="D87" s="4" t="inlineStr">
+      <c r="D87" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E87" s="4" t="inlineStr">
+      <c r="E87" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F87" s="4" t="inlineStr">
+      <c r="F87" s="11" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G87" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H87" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I87" s="4" t="n"/>
+      <c r="G87" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H87" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I87" s="11" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="4" t="n">
+      <c r="A88" s="11" t="n">
         <v>87</v>
       </c>
-      <c r="B88" s="4" t="inlineStr">
+      <c r="B88" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/103</t>
         </is>
       </c>
-      <c r="C88" s="4" t="inlineStr">
+      <c r="C88" s="11" t="inlineStr">
         <is>
           <t>3/26</t>
         </is>
       </c>
-      <c r="D88" s="4" t="inlineStr">
+      <c r="D88" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E88" s="4" t="inlineStr">
+      <c r="E88" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F88" s="4" t="inlineStr">
+      <c r="F88" s="11" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G88" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H88" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I88" s="4" t="n"/>
+      <c r="G88" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H88" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I88" s="11" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="4" t="n">
+      <c r="A89" s="11" t="n">
         <v>88</v>
       </c>
-      <c r="B89" s="4" t="inlineStr">
+      <c r="B89" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/104</t>
         </is>
       </c>
-      <c r="C89" s="4" t="inlineStr">
+      <c r="C89" s="11" t="inlineStr">
         <is>
           <t>4/26</t>
         </is>
       </c>
-      <c r="D89" s="4" t="inlineStr">
+      <c r="D89" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E89" s="4" t="inlineStr">
+      <c r="E89" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F89" s="4" t="inlineStr">
+      <c r="F89" s="11" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G89" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H89" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I89" s="4" t="n"/>
+      <c r="G89" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H89" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I89" s="11" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="4" t="n">
+      <c r="A90" s="11" t="n">
         <v>89</v>
       </c>
-      <c r="B90" s="4" t="inlineStr">
+      <c r="B90" s="11" t="inlineStr">
         <is>
           <t>FSL/2026/105</t>
         </is>
       </c>
-      <c r="C90" s="4" t="inlineStr">
+      <c r="C90" s="11" t="inlineStr">
         <is>
           <t>5/26</t>
         </is>
       </c>
-      <c r="D90" s="4" t="inlineStr">
+      <c r="D90" s="11" t="inlineStr">
         <is>
           <t>Sadar PS</t>
         </is>
       </c>
-      <c r="E90" s="4" t="inlineStr">
+      <c r="E90" s="11" t="inlineStr">
         <is>
           <t>376 IPC</t>
         </is>
       </c>
-      <c r="F90" s="4" t="inlineStr">
+      <c r="F90" s="11" t="inlineStr">
         <is>
           <t>Officer A</t>
         </is>
       </c>
-      <c r="G90" s="5" t="n">
-        <v>46135</v>
-      </c>
-      <c r="H90" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="I90" s="4" t="n"/>
+      <c r="G90" s="12" t="n">
+        <v>46135</v>
+      </c>
+      <c r="H90" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="I90" s="11" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -3965,37 +3977,37 @@
       <c r="I95" s="2" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="4" t="n">
+      <c r="A96" s="11" t="n">
         <v>93</v>
       </c>
-      <c r="B96" s="4" t="n"/>
-      <c r="C96" s="4" t="inlineStr">
+      <c r="B96" s="11" t="n"/>
+      <c r="C96" s="11" t="inlineStr">
         <is>
           <t>903/26</t>
         </is>
       </c>
-      <c r="D96" s="4" t="inlineStr">
+      <c r="D96" s="11" t="inlineStr">
         <is>
           <t>City PS</t>
         </is>
       </c>
-      <c r="E96" s="4" t="inlineStr">
+      <c r="E96" s="11" t="inlineStr">
         <is>
           <t>420 IPC</t>
         </is>
       </c>
-      <c r="F96" s="4" t="inlineStr">
+      <c r="F96" s="11" t="inlineStr">
         <is>
           <t>Officer Z</t>
         </is>
       </c>
-      <c r="G96" s="5" t="n">
-        <v>46140</v>
-      </c>
-      <c r="H96" s="5" t="n">
+      <c r="G96" s="12" t="n">
+        <v>46140</v>
+      </c>
+      <c r="H96" s="12" t="n">
         <v>46145</v>
       </c>
-      <c r="I96" s="4" t="n"/>
+      <c r="I96" s="11" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">

</xml_diff>